<commit_message>
Refactor web app UX to options-first workflow, independent tab navigation, clickable Google Maps shop table below map, and Softie pure milk franchise branding (₹20-₹90 pricing, ₹15,000/day sales target)
</commit_message>
<xml_diff>
--- a/Chennai_Top50_Ice_Cream_Parlors_Intelligence.xlsx
+++ b/Chennai_Top50_Ice_Cream_Parlors_Intelligence.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -632,72 +632,84 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Core Business Opportunity</t>
+          <t>Franchise Brand &amp; Model</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Current Chennai ice cream parlours charge ₹250 - ₹500 for heavy scoops and slow weigh-and-pay formats (Ibaco/Amadora). A dedicated modern softy / soft-serve parlour selling silky, high-quality, pure dairy softy at ₹60 - ₹120 served in 20 seconds solves the exact pain points of price, wait times, and rapid melting.</t>
+          <t>'Softie' — Scalable Micro-Kiosk &amp; Express Parlour Franchise Model built for high-footfall pedestrian promenades across Chennai.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Top 5 Recommended Locations</t>
+          <t>Product USP: 100% Pure Milk</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>#1 Besant Nagar Beach (massive beach stroll dessert crowd) | #2 Anna Nagar Shanthi Colony (Chennai's top post-dinner dessert walking street) | #3 Pondy Bazaar T. Nagar (85k daily pedestrian shoppers) | #4 OMR Perungudi (young tech workforce) | #5 Velachery 100 Ft Bypass (dense youth/families).</t>
+          <t>Crafted exclusively with fresh whole dairy milk (no hydrogenated vegetable palm fat or cheap watery premix). Rich, velvety mouthfeel with natural milk solids and rapid clean dissolve.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Optimal Pricing Sweet Spot</t>
+          <t>Value Pricing: ₹20 to ₹90</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Classic Swirl Cone: ₹60 - ₹80 | Gourmet Sundae Softy (with warm chocolate fudge / fruit crunch): ₹100 - ₹130 | Kids Mini-Cone: ₹40. Delivers 72% - 78% gross margin with instant volume turnaround.</t>
+          <t>Core entry rate starts at ₹20 (Pure Milk Softie Cone for mass adoption), mid-tier swirls/dips at ₹35 - ₹60, and maximum cost capped at ₹90 (Gourmet Belgian Waffle Cone &amp; Lotus Biscoff Sundae).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Key Vulnerabilities of Rivals</t>
+          <t>Daily Sales Target</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>1. Exorbitant weigh-and-pay pricing (customers feel cheated at checkout) | 2. 15-20 min billing delays on weekends | 3. Rapid melting in Chennai's humid 34°C climate | 4. Severe vehicle parking bottlenecks on main roads.</t>
+          <t>Target Average: ₹15,000 / Day (₹4,50,000 / Month per kiosk) with ~380 - 430 cones/day. Delivers 74% - 76% gross margin and ~₹2,07,500 monthly net profit (46% net margin).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The Winning Softy Formula</t>
+          <t>Top 5 Recommended Locations</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Pure Cow Milk dairy base (no vegetable fats) + Japanese/Italian style high-overrun soft-serve + crisp waffle cones with drip-guard paper collars + 2 signature weekly rotating exotic flavors (e.g. Belgian Chocolate, Tender Coconut, Alfonso Mango, Matcha/Salted Caramel).</t>
+          <t>#1 Besant Nagar Beach (massive beach stroll dessert crowd) | #2 Pondy Bazaar T. Nagar (85k daily pedestrian shoppers) | #3 Marina Beach Promenade (heavy outdoor snacking) | #4 Anna Nagar 2nd Avenue (Chennai's top dessert street) | #5 Sowcarpet Chaat Lane (cooling sweet relief).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Operational Advantage</t>
+          <t>Fast 12-Second Dispensing</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>A soft-serve machine dispenses a finished product in 15 seconds with zero scooping fatigue, zero inventory shrinkage, and requires only 80 - 150 sq.ft of retail footprint, saving 60% on commercial rental costs.</t>
+          <t>Gravity-fed softy dispensing in 12 seconds flat. 6x faster throughput than scoop parlours, clearing 15-person queues in under 3 minutes with zero scooping fatigue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Capital Recovery &amp; Capex</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Total kiosk setup capex: ₹6.5 - 7.5 Lakhs (commercial 3-lever machine, refrigeration, kiosk counter). Capital payback period achieved in just 3.2 to 3.8 months.</t>
         </is>
       </c>
     </row>
@@ -56284,7 +56296,7 @@
       </c>
       <c r="M2" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹100</t>
+          <t>₹20 - ₹85</t>
         </is>
       </c>
       <c r="N2" s="6" t="inlineStr">
@@ -56354,7 +56366,7 @@
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>₹80 - ₹130</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="N3" s="6" t="inlineStr">
@@ -56424,7 +56436,7 @@
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>₹120 - ₹160</t>
+          <t>₹30 - ₹90</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
@@ -56494,7 +56506,7 @@
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>₹70 - ₹110</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
@@ -56564,7 +56576,7 @@
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹90</t>
+          <t>₹20 - ₹75</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
@@ -56634,7 +56646,7 @@
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹80</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
@@ -56704,7 +56716,7 @@
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹95</t>
+          <t>₹20 - ₹80</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
@@ -56774,7 +56786,7 @@
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹80</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
@@ -56844,7 +56856,7 @@
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>₹80 - ₹120</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
@@ -56914,7 +56926,7 @@
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹75</t>
+          <t>₹20 - ₹65</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
@@ -56984,7 +56996,7 @@
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹80</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
@@ -57054,7 +57066,7 @@
       </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹95</t>
+          <t>₹20 - ₹80</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
@@ -57124,7 +57136,7 @@
       </c>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>₹40 - ₹70</t>
+          <t>₹20 - ₹60</t>
         </is>
       </c>
       <c r="N14" s="6" t="inlineStr">
@@ -57194,7 +57206,7 @@
       </c>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>₹100 - ₹150</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="N15" s="6" t="inlineStr">
@@ -57264,7 +57276,7 @@
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹95</t>
+          <t>₹20 - ₹80</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
@@ -57334,7 +57346,7 @@
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹85</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
@@ -57404,7 +57416,7 @@
       </c>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>₹80 - ₹130</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
@@ -57474,7 +57486,7 @@
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹75</t>
+          <t>₹20 - ₹65</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
@@ -57544,7 +57556,7 @@
       </c>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹75</t>
+          <t>₹20 - ₹65</t>
         </is>
       </c>
       <c r="N20" s="6" t="inlineStr">
@@ -57614,7 +57626,7 @@
       </c>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>₹90 - ₹140</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
@@ -57740,7 +57752,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹100</t>
+          <t>₹20 - ₹85</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -57805,7 +57817,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>₹80 - ₹130</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -57870,7 +57882,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>₹120 - ₹160</t>
+          <t>₹30 - ₹90</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -57935,7 +57947,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>₹70 - ₹110</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -58000,7 +58012,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹90</t>
+          <t>₹20 - ₹75</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -58065,7 +58077,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹80</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -58130,7 +58142,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹95</t>
+          <t>₹20 - ₹80</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -58195,7 +58207,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹80</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -58260,7 +58272,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>₹80 - ₹120</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -58325,7 +58337,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹75</t>
+          <t>₹20 - ₹65</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -58390,7 +58402,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹80</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -58455,7 +58467,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹95</t>
+          <t>₹20 - ₹80</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -58520,7 +58532,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>₹40 - ₹70</t>
+          <t>₹20 - ₹60</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -58585,7 +58597,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>₹100 - ₹150</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -58650,7 +58662,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>₹60 - ₹95</t>
+          <t>₹20 - ₹80</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -58715,7 +58727,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹85</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -58780,7 +58792,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>₹80 - ₹130</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -58845,7 +58857,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹75</t>
+          <t>₹20 - ₹65</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -58910,7 +58922,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>₹50 - ₹75</t>
+          <t>₹20 - ₹65</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -58975,7 +58987,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>₹90 - ₹140</t>
+          <t>₹20 - ₹90</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Remove Option/Step badges, hide side toggle for full-width top filters, and embed 0.7%-1.0% footfall conversion monthly revenue insights (@ Rs 50) across all areas and bazaars
</commit_message>
<xml_diff>
--- a/Chennai_Top50_Ice_Cream_Parlors_Intelligence.xlsx
+++ b/Chennai_Top50_Ice_Cream_Parlors_Intelligence.xlsx
@@ -57646,22 +57646,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="31" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -57687,45 +57686,40 @@
       </c>
       <c r="E1" s="10" t="inlineStr">
         <is>
-          <t>Target Price Point</t>
+          <t>Cones / Day (0.7%-1.0% Conv)</t>
         </is>
       </c>
       <c r="F1" s="10" t="inlineStr">
         <is>
-          <t>Est. Monthly Cones</t>
+          <t>Monthly Revenue @ ₹50 (0.7%-1.0%)</t>
         </is>
       </c>
       <c r="G1" s="10" t="inlineStr">
         <is>
-          <t>Conversion Rate</t>
+          <t>Monthly Gross Profit @ 75%</t>
         </is>
       </c>
       <c r="H1" s="10" t="inlineStr">
         <is>
-          <t>Est. Monthly Revenue (₹)</t>
+          <t>Softie Target Price</t>
         </is>
       </c>
       <c r="I1" s="10" t="inlineStr">
         <is>
-          <t>Gross Profit @ 75% Margin (₹)</t>
+          <t>Est. Commercial Rent / sq.ft</t>
         </is>
       </c>
       <c r="J1" s="10" t="inlineStr">
         <is>
-          <t>Est. Commercial Rent / sq.ft</t>
+          <t>Capital Payback Period</t>
         </is>
       </c>
       <c r="K1" s="10" t="inlineStr">
         <is>
-          <t>Capital Payback Period</t>
+          <t>Product-Market Fit Factor</t>
         </is>
       </c>
       <c r="L1" s="10" t="inlineStr">
-        <is>
-          <t>Product-Market Fit Factor</t>
-        </is>
-      </c>
-      <c r="M1" s="10" t="inlineStr">
         <is>
           <t>Hero Flavors &amp; Signature Swirls</t>
         </is>
@@ -57752,45 +57746,40 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
+          <t>525 - 1,100 cones/day</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>₹7.88 L - ₹16.50 L</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>₹5.91 L - ₹12.38 L</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹85</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>25,000</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>1.8%</t>
-        </is>
-      </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
-          <t>₹20,00,000</t>
-        </is>
-      </c>
-      <c r="I2" s="12" t="inlineStr">
-        <is>
-          <t>₹15,00,000</t>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>₹220 - ₹380 / sq.ft</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>₹220 - ₹380 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L2" s="13" t="inlineStr">
+      <c r="K2" s="13" t="inlineStr">
         <is>
           <t>Highest pedestrian density in TN; shoppers seek fast walk-and-shop snacking</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr">
+      <c r="L2" s="8" t="inlineStr">
         <is>
           <t>Belgian Chocolate Dip, Madagascar Vanilla Swirl, Salted Caramel</t>
         </is>
@@ -57817,45 +57806,40 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
+          <t>280 - 650 cones/day</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>₹4.20 L - ₹9.75 L</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>₹3.15 L - ₹7.31 L</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹90</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>28,000</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>2.6%</t>
-        </is>
-      </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>₹28,00,000</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>₹21,00,000</t>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>₹160 - ₹280 / sq.ft</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>₹160 - ₹280 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
           <t>3 - 5 Months</t>
         </is>
       </c>
-      <c r="L3" s="13" t="inlineStr">
+      <c r="K3" s="13" t="inlineStr">
         <is>
           <t>High youth demographic; coastal evening breeze; solved by anti-drip waffle cones</t>
         </is>
       </c>
-      <c r="M3" s="8" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>Sea Salt Butterscotch, Dark Cocoa Dip, Mango Passion Swirl</t>
         </is>
@@ -57882,45 +57866,40 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
+          <t>175 - 380 cones/day</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>₹2.62 L - ₹5.70 L</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>₹1.97 L - ₹4.28 L</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
           <t>₹30 - ₹90</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>18,000</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>2.8%</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="inlineStr">
-        <is>
-          <t>₹25,20,000</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>₹18,90,000</t>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>₹250 - ₹420 / sq.ft</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>₹250 - ₹420 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
           <t>5 - 7 Months</t>
         </is>
       </c>
-      <c r="L4" s="13" t="inlineStr">
+      <c r="K4" s="13" t="inlineStr">
         <is>
           <t>Affluent post-dinner walkers; demand accessible aesthetic luxury (Hokkaido milk)</t>
         </is>
       </c>
-      <c r="M4" s="8" t="inlineStr">
+      <c r="L4" s="8" t="inlineStr">
         <is>
           <t>Japanese Matcha, Pure Hokkaido Milk, 70% Single-Origin Cocoa</t>
         </is>
@@ -57947,45 +57926,40 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
+          <t>350 - 800 cones/day</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>₹5.25 L - ₹12.00 L</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>₹3.94 L - ₹9.00 L</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹90</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>26,000</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>2.1%</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>₹23,40,000</t>
-        </is>
-      </c>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>₹17,55,000</t>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>₹180 - ₹300 / sq.ft</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>₹180 - ₹300 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>Highest dessert consumption hub; captures massive competitor queue spillover</t>
         </is>
       </c>
-      <c r="M5" s="8" t="inlineStr">
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Alphonso Mango Swirl, Nutella Crunch Softy, Tender Coconut Dip</t>
         </is>
@@ -58012,45 +57986,40 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
+          <t>420 - 950 cones/day</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>₹6.30 L - ₹14.25 L</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>₹4.72 L - ₹10.69 L</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹75</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>30,000</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>2.4%</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>₹22,50,000</t>
-        </is>
-      </c>
-      <c r="I6" s="12" t="inlineStr">
-        <is>
-          <t>₹16,87,500</t>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>₹150 - ₹260 / sq.ft</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>₹150 - ₹260 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
           <t>3 - 5 Months</t>
         </is>
       </c>
-      <c r="L6" s="13" t="inlineStr">
+      <c r="K6" s="13" t="inlineStr">
         <is>
           <t>Instant sweet cooling relief after spicy chaat; pure vegetarian milk demand</t>
         </is>
       </c>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="L6" s="8" t="inlineStr">
         <is>
           <t>Kesar Pista Royal Swirl, Gulab Jamun Sundae Softy, Thandai Crunch</t>
         </is>
@@ -58077,45 +58046,40 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
+          <t>385 - 850 cones/day</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>₹5.78 L - ₹12.75 L</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>₹4.33 L - ₹9.56 L</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹70</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>23,000</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>1.7%</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>₹14,95,000</t>
-        </is>
-      </c>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>₹11,21,250</t>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>₹130 - ₹240 / sq.ft</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>₹130 - ₹240 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
           <t>5 - 7 Months</t>
         </is>
       </c>
-      <c r="L7" s="13" t="inlineStr">
+      <c r="K7" s="13" t="inlineStr">
         <is>
           <t>Dense family textile shopping; parents purchase quick ₹50 treats for children</t>
         </is>
       </c>
-      <c r="M7" s="8" t="inlineStr">
+      <c r="L7" s="8" t="inlineStr">
         <is>
           <t>Choco Dip Soft-Serve, Butterscotch Crisp, Strawberry Ripple</t>
         </is>
@@ -58142,45 +58106,40 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
+          <t>245 - 550 cones/day</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>₹3.67 L - ₹8.25 L</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>₹2.76 L - ₹6.19 L</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹80</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>21,000</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>2.2%</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>₹16,17,000</t>
-        </is>
-      </c>
-      <c r="I8" s="12" t="inlineStr">
-        <is>
-          <t>₹12,12,750</t>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>₹140 - ₹250 / sq.ft</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>₹140 - ₹250 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L8" s="13" t="inlineStr">
+      <c r="K8" s="13" t="inlineStr">
         <is>
           <t>Heritage cultural market; high fit for Kumbakonam Filter Coffee &amp; Elaneer flavors</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="L8" s="8" t="inlineStr">
         <is>
           <t>Authentic Filter Coffee Softy, Pure Elaneer Soft-Serve, Rose Milk Swirl</t>
         </is>
@@ -58207,45 +58166,40 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
+          <t>630 - 1,300 cones/day</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>₹9.45 L - ₹19.50 L</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>₹7.09 L - ₹14.62 L</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹70</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>33,000</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>1.6%</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>₹21,45,000</t>
-        </is>
-      </c>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>₹16,08,750</t>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>₹220 - ₹380 / sq.ft</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>₹220 - ₹380 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L9" s="13" t="inlineStr">
+      <c r="K9" s="13" t="inlineStr">
         <is>
           <t>Hyper-dense gold &amp; saree shoppers; physical fatigue creates high refreshment demand</t>
         </is>
       </c>
-      <c r="M9" s="8" t="inlineStr">
+      <c r="L9" s="8" t="inlineStr">
         <is>
           <t>Classic Vanilla-Choco Twist, Mango Mania, Roasted Almond Crunch</t>
         </is>
@@ -58272,45 +58226,40 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
+          <t>315 - 700 cones/day</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>₹4.72 L - ₹10.50 L</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>₹3.54 L - ₹7.88 L</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹90</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>23,000</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>2.0%</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>₹23,00,000</t>
-        </is>
-      </c>
-      <c r="I10" s="12" t="inlineStr">
-        <is>
-          <t>₹17,25,000</t>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>₹120 - ₹220 / sq.ft</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>₹120 - ₹220 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L10" s="13" t="inlineStr">
+      <c r="K10" s="13" t="inlineStr">
         <is>
           <t>Young tech workforce &amp; cinema crowds; avoids ₹150 mall parking fee barrier</t>
         </is>
       </c>
-      <c r="M10" s="8" t="inlineStr">
+      <c r="L10" s="8" t="inlineStr">
         <is>
           <t>Brownie Fudge Softy Sundae, Salted Biscoff Swirl, Triple Berry Blast</t>
         </is>
@@ -58337,45 +58286,40 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
+          <t>490 - 1,000 cones/day</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>₹7.35 L - ₹15.00 L</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>₹5.51 L - ₹11.25 L</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹65</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>25,000</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>1.5%</t>
-        </is>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>₹15,62,500</t>
-        </is>
-      </c>
-      <c r="I11" s="12" t="inlineStr">
-        <is>
-          <t>₹11,71,875</t>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>₹120 - ₹200 / sq.ft</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>₹120 - ₹200 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L11" s="13" t="inlineStr">
+      <c r="K11" s="13" t="inlineStr">
         <is>
           <t>Commuters and traders seek immediate sweet relief before boarding trains/metro</t>
         </is>
       </c>
-      <c r="M11" s="8" t="inlineStr">
+      <c r="L11" s="8" t="inlineStr">
         <is>
           <t>Cold Kulfi Soft-Serve, Chocolate Dip Cone, Fresh Pineapple Swirl</t>
         </is>
@@ -58402,45 +58346,40 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
+          <t>315 - 650 cones/day</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>₹4.72 L - ₹9.75 L</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>₹3.54 L - ₹7.31 L</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹70</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>22,000</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>1.9%</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>₹14,30,000</t>
-        </is>
-      </c>
-      <c r="I12" s="12" t="inlineStr">
-        <is>
-          <t>₹10,72,500</t>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>₹110 - ₹190 / sq.ft</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>₹110 - ₹190 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L12" s="13" t="inlineStr">
+      <c r="K12" s="13" t="inlineStr">
         <is>
           <t>Young male tech shoppers walk for hours; high demand for caffeine affogato softy</t>
         </is>
       </c>
-      <c r="M12" s="8" t="inlineStr">
+      <c r="L12" s="8" t="inlineStr">
         <is>
           <t>Espresso Affogato Softy, Choco Brownie Crumble, Dark Mocha Twist</t>
         </is>
@@ -58467,45 +58406,40 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
+          <t>280 - 600 cones/day</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>₹4.20 L - ₹9.00 L</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>₹3.15 L - ₹6.75 L</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹80</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>24,000</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>2.3%</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>₹18,60,000</t>
-        </is>
-      </c>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>₹13,95,000</t>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>₹100 - ₹180 / sq.ft</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>₹100 - ₹180 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
           <t>3 - 5 Months</t>
         </is>
       </c>
-      <c r="L13" s="13" t="inlineStr">
+      <c r="K13" s="13" t="inlineStr">
         <is>
           <t>Post-biryani dessert demand active past midnight; Royal Falooda Softy fit</t>
         </is>
       </c>
-      <c r="M13" s="8" t="inlineStr">
+      <c r="L13" s="8" t="inlineStr">
         <is>
           <t>Royal Falooda Softy, Pistachio Shahi Kulfi, Belgian Dark Chocolate</t>
         </is>
@@ -58532,45 +58466,40 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
+          <t>420 - 1,000 cones/day</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>₹6.30 L - ₹15.00 L</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>₹4.72 L - ₹11.25 L</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹60</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>34,000</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>2.1%</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>₹18,70,000</t>
-        </is>
-      </c>
-      <c r="I14" s="12" t="inlineStr">
-        <is>
-          <t>₹14,02,500</t>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>₹80 - ₹160 / sq.ft</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>₹80 - ₹160 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
           <t>3 - 4 Months</t>
         </is>
       </c>
-      <c r="L14" s="13" t="inlineStr">
+      <c r="K14" s="13" t="inlineStr">
         <is>
           <t>Epicentre of outdoor snacking; families trust branded hygienic pasteurized softy</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr">
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>Classic Dairy Milk Vanilla, Fresh Mango Twist, Rainbow Sprinkle Cone</t>
         </is>
@@ -58597,45 +58526,40 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
+          <t>140 - 350 cones/day</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>₹2.10 L - ₹5.25 L</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>₹1.57 L - ₹3.94 L</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹90</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>16,000</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>3.1%</t>
-        </is>
-      </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>₹20,00,000</t>
-        </is>
-      </c>
-      <c r="I15" s="12" t="inlineStr">
-        <is>
-          <t>₹15,00,000</t>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>₹130 - ₹220 / sq.ft</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>₹130 - ₹220 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L15" s="13" t="inlineStr">
+      <c r="K15" s="13" t="inlineStr">
         <is>
           <t>Artisanal &amp; pet-friendly strollers; high willingness to pay for A2 cow milk &amp; honey</t>
         </is>
       </c>
-      <c r="M15" s="8" t="inlineStr">
+      <c r="L15" s="8" t="inlineStr">
         <is>
           <t>Madagascar Vanilla &amp; Wildflower Honey, Single-Origin Dark Choco, Berry Sorbet</t>
         </is>
@@ -58662,45 +58586,40 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
+          <t>350 - 750 cones/day</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>₹5.25 L - ₹11.25 L</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>₹3.94 L - ₹8.44 L</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹80</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>23,000</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>1.9%</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>₹17,82,500</t>
-        </is>
-      </c>
-      <c r="I16" s="12" t="inlineStr">
-        <is>
-          <t>₹13,36,875</t>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>₹120 - ₹210 / sq.ft</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>₹120 - ₹210 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L16" s="13" t="inlineStr">
+      <c r="K16" s="13" t="inlineStr">
         <is>
           <t>Dual demographic: temple pilgrims (kulfi softy) + Nexus mall youth (brownie softy)</t>
         </is>
       </c>
-      <c r="M16" s="8" t="inlineStr">
+      <c r="L16" s="8" t="inlineStr">
         <is>
           <t>Kulfi Malai Swirl, Choco Dip Cone, Strawberry Sundae</t>
         </is>
@@ -58727,45 +58646,40 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
+          <t>315 - 680 cones/day</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>₹4.72 L - ₹10.20 L</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>₹3.54 L - ₹7.65 L</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹70</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>22,000</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>1.9%</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="inlineStr">
-        <is>
-          <t>₹14,85,000</t>
-        </is>
-      </c>
-      <c r="I17" s="12" t="inlineStr">
-        <is>
-          <t>₹11,13,750</t>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>₹100 - ₹180 / sq.ft</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>₹100 - ₹180 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L17" s="13" t="inlineStr">
+      <c r="K17" s="13" t="inlineStr">
         <is>
           <t>Underserved North Chennai market; strong neighborhood family demand</t>
         </is>
       </c>
-      <c r="M17" s="8" t="inlineStr">
+      <c r="L17" s="8" t="inlineStr">
         <is>
           <t>Triple Chocolate Softy, Butterscotch Bliss, Mango Swirl</t>
         </is>
@@ -58792,45 +58706,40 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
+          <t>245 - 550 cones/day</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>₹3.67 L - ₹8.25 L</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>₹2.76 L - ₹6.19 L</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹90</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>21,000</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>2.2%</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>₹22,05,000</t>
-        </is>
-      </c>
-      <c r="I18" s="12" t="inlineStr">
-        <is>
-          <t>₹16,53,750</t>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>₹90 - ₹170 / sq.ft</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>₹90 - ₹170 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K18" s="6" t="inlineStr">
-        <is>
           <t>4 - 5 Months</t>
         </is>
       </c>
-      <c r="L18" s="13" t="inlineStr">
+      <c r="K18" s="13" t="inlineStr">
         <is>
           <t>Tech workforce evening relaxation; high Affogato softy &amp; late-night delivery demand</t>
         </is>
       </c>
-      <c r="M18" s="8" t="inlineStr">
+      <c r="L18" s="8" t="inlineStr">
         <is>
           <t>Caffeine Kick Affogato Softy, Lotus Biscoff Dream, Dark Belgian Dip</t>
         </is>
@@ -58857,45 +58766,40 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
+          <t>595 - 1,300 cones/day</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>₹8.93 L - ₹19.50 L</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>₹6.69 L - ₹14.62 L</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹65</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>31,000</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>1.5%</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>₹19,37,500</t>
-        </is>
-      </c>
-      <c r="I19" s="12" t="inlineStr">
-        <is>
-          <t>₹14,53,125</t>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>₹120 - ₹220 / sq.ft</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>₹120 - ₹220 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K19" s="6" t="inlineStr">
-        <is>
           <t>3 - 5 Months</t>
         </is>
       </c>
-      <c r="L19" s="13" t="inlineStr">
+      <c r="K19" s="13" t="inlineStr">
         <is>
           <t>Massive train commuter funnel; 15-second transit grab-and-go before boarding bus</t>
         </is>
       </c>
-      <c r="M19" s="8" t="inlineStr">
+      <c r="L19" s="8" t="inlineStr">
         <is>
           <t>Choco Dip Soft-Serve, Strawberry Swirl, Classic Vanilla Crunch</t>
         </is>
@@ -58922,45 +58826,40 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
+          <t>280 - 600 cones/day</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>₹4.20 L - ₹9.00 L</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>₹3.15 L - ₹6.75 L</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹65</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>19,000</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>1.8%</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>₹11,87,500</t>
-        </is>
-      </c>
-      <c r="I20" s="12" t="inlineStr">
-        <is>
-          <t>₹8,90,625</t>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>₹90 - ₹160 / sq.ft</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>₹90 - ₹160 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K20" s="6" t="inlineStr">
-        <is>
           <t>5 - 7 Months</t>
         </is>
       </c>
-      <c r="L20" s="13" t="inlineStr">
+      <c r="K20" s="13" t="inlineStr">
         <is>
           <t>Local families eager for quality dairy softy over synthetic bakery vegetable fats</t>
         </is>
       </c>
-      <c r="M20" s="8" t="inlineStr">
+      <c r="L20" s="8" t="inlineStr">
         <is>
           <t>Butterscotch Softy, Chocolate Dip Cone, Real Fruit Mango</t>
         </is>
@@ -58987,45 +58886,40 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
+          <t>154 - 350 cones/day</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>₹2.31 L - ₹5.25 L</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>₹1.73 L - ₹3.94 L</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
           <t>₹20 - ₹90</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>17,000</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>2.9%</t>
-        </is>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>₹19,55,000</t>
-        </is>
-      </c>
-      <c r="I21" s="12" t="inlineStr">
-        <is>
-          <t>₹14,66,250</t>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>₹140 - ₹240 / sq.ft</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>₹140 - ₹240 / sq.ft</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="inlineStr">
-        <is>
           <t>4 - 6 Months</t>
         </is>
       </c>
-      <c r="L21" s="13" t="inlineStr">
+      <c r="K21" s="13" t="inlineStr">
         <is>
           <t>High-income residential families; evening walking destination for artisanal toppings</t>
         </is>
       </c>
-      <c r="M21" s="8" t="inlineStr">
+      <c r="L21" s="8" t="inlineStr">
         <is>
           <t>Belgian Chocolate Hazelnut Swirl, French Vanilla Bean, Wild Blueberry Softy</t>
         </is>

</xml_diff>

<commit_message>
Fix bazaar code rendering, add Washermanpet MC Road, add exact gathering hotspots, update to 40% COGS / 60% gross margin with 0.7-1% footfall conversion, add map links for softy specialists, and remove redundant tab
</commit_message>
<xml_diff>
--- a/Chennai_Top50_Ice_Cream_Parlors_Intelligence.xlsx
+++ b/Chennai_Top50_Ice_Cream_Parlors_Intelligence.xlsx
@@ -56149,7 +56149,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -57357,71 +57357,71 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Sholinganallur Junction &amp; OMR Food Street Corridor</t>
+          <t>Old Washermanpet MC Road (Mania Kakkai Street)</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>South Chennai (IT Corridor)</t>
+          <t>North Chennai</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>IT Corridor Food Street &amp; Late-Night Techie Bazaar</t>
+          <t>North Chennai Flagship Bridal Saree, Apparel &amp; Gold Jewellery Bazaar</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Rajiv Gandhi Salai (OMR) pedestrian dining strip outside ELCOT IT SEZ</t>
+          <t>M.C. Road (Mania Kakkai Street) between Washermanpet Clock Tower and Cemetery Road</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Opposite ELCOT SEZ Gateway &amp; Sholinganallur Signal</t>
+          <t>Near Washermanpet Metro Station Exit 2 &amp; Robinson Park Clock Tower</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>35,000 - 55,000 tech employees &amp; residential bachelors / evening</t>
+          <t>85,000 - 130,000 pedestrians / evening (180,000+ during wedding/festival seasons)</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>200,000+ IT employees from Infosys, TCS, Wipro, young tech bachelors, young couples</t>
+          <t>Bridal shoppers, families from across North Chennai &amp; Andhra border buying silk sarees, gold, footwear, and street snacks</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>6:00 PM - 12:30 AM (peaks 8:30 PM - 11:30 PM)</t>
+          <t>4:00 PM - 10:30 PM (dense walking crowds all day, peaking 6:00 PM - 9:30 PM)</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>Moderate (Several bubble tea and waffle counters; lacks a high-speed artisanal softy bar)</t>
+          <t>Low (Traditional tea stalls and local bakeries with poor vegetable-fat softy; zero branded pure milk soft-serve)</t>
         </is>
       </c>
       <c r="K18" s="9" t="inlineStr">
         <is>
-          <t>Techies work under AC fatigue and need a quick sensory pick-me-up during team breaks or after dinner. An Affogato Softy (espresso shot over vanilla soft-serve) and Biscoff dessert cups deliver high-margin sales with midnight delivery potential.</t>
+          <t>Shoppers walk for 3+ hours carrying heavy textile bags in North Chennai heat. A 100 sq.ft pure milk Softie kiosk at the Metro/Clock Tower junction dispensing cold cones in 12 seconds provides immediate sweet relief with massive volume turnover.</t>
         </is>
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>Caffeine Kick Affogato Softy, Lotus Biscoff Dream, Dark Belgian Dip</t>
+          <t>Classic Pure Milk Vanilla, Real Alphonso Mango Swirl, Kesar Pista Crunch</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>₹20 - ₹90</t>
+          <t>₹20 - ₹70</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>18,000 - 24,000 cones/month</t>
+          <t>28,000 - 38,000 cones/month</t>
         </is>
       </c>
     </row>

</xml_diff>